<commit_message>
Updated TODOs, exctracted sample preparation logic to a separate method
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/data/european_offshore_wind_capex.xlsx
+++ b/data/european_offshore_wind_capex.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weron\Pulpit\sem3\ds_workshop\WindFarm\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17E1E4A1-7783-4DC4-A1E7-7583DA59EF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F86846-A451-40C2-85C3-D990FB56EBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="30912" windowHeight="18672" xr2:uid="{D4FCA4BE-944B-479A-AF27-5DDC1E18E177}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{D4FCA4BE-944B-479A-AF27-5DDC1E18E177}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3104,9 +3104,6 @@
     <t>25,9</t>
   </si>
   <si>
-    <t>area</t>
-  </si>
-  <si>
     <t>41.3</t>
   </si>
   <si>
@@ -3174,6 +3171,9 @@
   </si>
   <si>
     <t>247</t>
+  </si>
+  <si>
+    <t>area_sqkm</t>
   </si>
 </sst>
 </file>
@@ -3641,7 +3641,7 @@
         <v>845</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1014</v>
+        <v>1037</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -6455,7 +6455,7 @@
         <v>881</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="E40" s="5" t="s">
         <v>22</v>
@@ -6819,7 +6819,7 @@
         <v>886</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>22</v>
@@ -6967,7 +6967,7 @@
         <v>888</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>22</v>
@@ -7041,7 +7041,7 @@
         <v>924</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>22</v>
@@ -7411,7 +7411,7 @@
         <v>891</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>280</v>
@@ -7559,7 +7559,7 @@
         <v>927</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>280</v>
@@ -7855,7 +7855,7 @@
         <v>892</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>280</v>
@@ -8077,7 +8077,7 @@
         <v>932</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>280</v>
@@ -8447,7 +8447,7 @@
         <v>895</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>280</v>
@@ -8595,7 +8595,7 @@
         <v>897</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>280</v>
@@ -8669,7 +8669,7 @@
         <v>898</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>280</v>
@@ -8817,7 +8817,7 @@
         <v>899</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>280</v>
@@ -9187,7 +9187,7 @@
         <v>902</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="E77" s="1" t="s">
         <v>280</v>
@@ -9261,7 +9261,7 @@
         <v>903</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>280</v>
@@ -9335,7 +9335,7 @@
         <v>904</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="E79" s="1" t="s">
         <v>280</v>
@@ -9409,7 +9409,7 @@
         <v>905</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>280</v>
@@ -9853,7 +9853,7 @@
         <v>940</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="E86" s="1" t="s">
         <v>408</v>
@@ -9927,7 +9927,7 @@
         <v>907</v>
       </c>
       <c r="D87" s="5" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="E87" s="5" t="s">
         <v>408</v>
@@ -10001,7 +10001,7 @@
         <v>908</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="E88" s="1" t="s">
         <v>408</v>
@@ -10149,7 +10149,7 @@
         <v>910</v>
       </c>
       <c r="D90" s="5" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="E90" s="5" t="s">
         <v>408</v>
@@ -10223,7 +10223,7 @@
         <v>911</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="E91" s="1" t="s">
         <v>408</v>
@@ -10371,7 +10371,7 @@
         <v>912</v>
       </c>
       <c r="D93" s="5" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="E93" s="5" t="s">
         <v>408</v>
@@ -10741,7 +10741,7 @@
         <v>927</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="E98" s="1" t="s">
         <v>408</v>
@@ -10815,7 +10815,7 @@
         <v>942</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="E99" s="1" t="s">
         <v>408</v>
@@ -11037,7 +11037,7 @@
         <v>927</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="E102" s="1" t="s">
         <v>408</v>
@@ -11185,7 +11185,7 @@
         <v>944</v>
       </c>
       <c r="D104" s="5" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="E104" s="5" t="s">
         <v>408</v>
@@ -11333,7 +11333,7 @@
         <v>920</v>
       </c>
       <c r="D106" s="5" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="E106" s="5" t="s">
         <v>497</v>
@@ -11407,7 +11407,7 @@
         <v>921</v>
       </c>
       <c r="D107" s="5" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="E107" s="5" t="s">
         <v>497</v>

</xml_diff>

<commit_message>
Filled missing installed capaciity and distance from shore
</commit_message>
<xml_diff>
--- a/data/european_offshore_wind_capex.xlsx
+++ b/data/european_offshore_wind_capex.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weron\Pulpit\sem3\ds_workshop\WindFarm\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F86846-A451-40C2-85C3-D990FB56EBF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C07962A8-B80E-4C3F-B87F-08A04A07C6D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{D4FCA4BE-944B-479A-AF27-5DDC1E18E177}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4207" uniqueCount="1038">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4207" uniqueCount="1046">
   <si>
     <t>wind_farm_name</t>
   </si>
@@ -3174,6 +3174,30 @@
   </si>
   <si>
     <t>area_sqkm</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>85-96</t>
+  </si>
+  <si>
+    <t>140-214</t>
+  </si>
+  <si>
+    <t>77-102</t>
+  </si>
+  <si>
+    <t>77</t>
+  </si>
+  <si>
+    <t>10-25</t>
+  </si>
+  <si>
+    <t>600-900</t>
+  </si>
+  <si>
+    <t>10-15</t>
   </si>
 </sst>
 </file>
@@ -4382,7 +4406,7 @@
         <v>36</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>30</v>
+        <v>110</v>
       </c>
       <c r="L11" s="4" t="s">
         <v>30</v>
@@ -5606,7 +5630,7 @@
         <v>30</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>30</v>
+        <v>1038</v>
       </c>
       <c r="L28" s="4" t="s">
         <v>30</v>
@@ -5678,7 +5702,7 @@
         <v>169</v>
       </c>
       <c r="K29" s="4" t="s">
-        <v>30</v>
+        <v>216</v>
       </c>
       <c r="L29" s="5" t="s">
         <v>170</v>
@@ -9726,7 +9750,7 @@
         <v>30</v>
       </c>
       <c r="K84" s="4" t="s">
-        <v>30</v>
+        <v>1039</v>
       </c>
       <c r="L84" s="5" t="s">
         <v>403</v>
@@ -10392,7 +10416,7 @@
         <v>449</v>
       </c>
       <c r="K93" s="4" t="s">
-        <v>30</v>
+        <v>175</v>
       </c>
       <c r="L93" s="4" t="s">
         <v>30</v>
@@ -11132,7 +11156,7 @@
         <v>30</v>
       </c>
       <c r="K103" s="4" t="s">
-        <v>30</v>
+        <v>180</v>
       </c>
       <c r="L103" s="4" t="s">
         <v>30</v>
@@ -11794,7 +11818,7 @@
         <v>30</v>
       </c>
       <c r="K112" s="4" t="s">
-        <v>30</v>
+        <v>267</v>
       </c>
       <c r="L112" s="4" t="s">
         <v>30</v>
@@ -11866,7 +11890,7 @@
         <v>30</v>
       </c>
       <c r="K113" s="4" t="s">
-        <v>30</v>
+        <v>1040</v>
       </c>
       <c r="L113" s="4" t="s">
         <v>30</v>
@@ -12010,7 +12034,7 @@
         <v>30</v>
       </c>
       <c r="K115" s="4" t="s">
-        <v>30</v>
+        <v>216</v>
       </c>
       <c r="L115" s="5" t="s">
         <v>535</v>
@@ -13378,7 +13402,7 @@
         <v>30</v>
       </c>
       <c r="K134" s="4" t="s">
-        <v>30</v>
+        <v>1041</v>
       </c>
       <c r="L134" s="4" t="s">
         <v>30</v>
@@ -13450,7 +13474,7 @@
         <v>30</v>
       </c>
       <c r="K135" s="4" t="s">
-        <v>30</v>
+        <v>1042</v>
       </c>
       <c r="L135" s="4" t="s">
         <v>30</v>
@@ -14170,7 +14194,7 @@
         <v>30</v>
       </c>
       <c r="K145" s="4" t="s">
-        <v>30</v>
+        <v>325</v>
       </c>
       <c r="L145" s="4" t="s">
         <v>30</v>
@@ -14242,7 +14266,7 @@
         <v>30</v>
       </c>
       <c r="K146" s="4" t="s">
-        <v>30</v>
+        <v>325</v>
       </c>
       <c r="L146" s="4" t="s">
         <v>30</v>
@@ -15598,7 +15622,7 @@
         <v>66</v>
       </c>
       <c r="G165" s="4" t="s">
-        <v>30</v>
+        <v>1044</v>
       </c>
       <c r="H165" s="5" t="s">
         <v>30</v>
@@ -15610,7 +15634,7 @@
         <v>30</v>
       </c>
       <c r="K165" s="4" t="s">
-        <v>30</v>
+        <v>1043</v>
       </c>
       <c r="L165" s="4" t="s">
         <v>30</v>
@@ -15898,7 +15922,7 @@
         <v>30</v>
       </c>
       <c r="K169" s="4" t="s">
-        <v>30</v>
+        <v>615</v>
       </c>
       <c r="L169" s="5" t="s">
         <v>693</v>
@@ -15958,7 +15982,7 @@
         <v>30</v>
       </c>
       <c r="G170" s="4" t="s">
-        <v>30</v>
+        <v>397</v>
       </c>
       <c r="H170" s="5" t="s">
         <v>30</v>
@@ -15970,7 +15994,7 @@
         <v>30</v>
       </c>
       <c r="K170" s="4" t="s">
-        <v>30</v>
+        <v>734</v>
       </c>
       <c r="L170" s="4" t="s">
         <v>30</v>
@@ -16186,7 +16210,7 @@
         <v>30</v>
       </c>
       <c r="K173" s="4" t="s">
-        <v>30</v>
+        <v>551</v>
       </c>
       <c r="L173" s="4" t="s">
         <v>30</v>
@@ -16546,7 +16570,7 @@
         <v>30</v>
       </c>
       <c r="K178" s="4" t="s">
-        <v>30</v>
+        <v>233</v>
       </c>
       <c r="L178" s="4" t="s">
         <v>30</v>
@@ -16906,7 +16930,7 @@
         <v>30</v>
       </c>
       <c r="K183" s="4" t="s">
-        <v>30</v>
+        <v>1045</v>
       </c>
       <c r="L183" s="4" t="s">
         <v>30</v>

</xml_diff>